<commit_message>
Anomalies SF1-RTSP — 25/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF1-RTSP/anomalies.xlsx
+++ b/presentation/SF1-RTSP/anomalies.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2143,10 +2143,10 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>12073718</v>
+        <v>12073715</v>
       </c>
       <c r="B20" t="n">
-        <v>4001211814</v>
+        <v>4001211811</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2155,24 +2155,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>OR004001211814</t>
+          <t>OR004001211811</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-REACTI-0CA208-SURV-PI2084</t>
+          <t>SF01-PE-00LS-REACTI-0CA208-SURV-PI2083</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>MANOMETRE VAPEUR D'INJECTEUR 4 CA</t>
+          <t>MANOMETRE VAPEUR D'INJECTEUR 3 CA</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>S-PC-PI2084</t>
+          <t>S-PC-PI2083</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="Q20" s="2" t="n">
         <v>46062</v>
@@ -2232,10 +2232,10 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>12073720</v>
+        <v>12073718</v>
       </c>
       <c r="B21" t="n">
-        <v>4001211820</v>
+        <v>4001211814</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2244,24 +2244,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>OR004001211820</t>
+          <t>OR004001211814</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-GRANUL-0HB138-SURV-B138</t>
+          <t>SF01-PE-00LS-REACTI-0CA208-SURV-PI2084</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BOBINE DISTRIB CENTRALE HYDRO COUTEAU</t>
+          <t>MANOMETRE VAPEUR D'INJECTEUR 4 CA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>S-PC-B138</t>
+          <t>S-PC-PI2084</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2320,35 +2320,37 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="n">
+        <v>12073720</v>
+      </c>
       <c r="B22" t="n">
-        <v>4001211902</v>
+        <v>4001211820</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>REVISION DETENDEUR</t>
+          <t>PREVENTIF SYSTEMATIQUE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>OR004001211902</t>
+          <t>OR004001211820</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-PRV7012</t>
+          <t>SF01-PE-00LS-GRANUL-0HB138-SURV-B138</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>REGULATEUR PRESSION FUEL ENTRÈE BRULEUR</t>
+          <t>BOBINE DISTRIB CENTRALE HYDRO COUTEAU</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>S-PC-PRV7012</t>
+          <t>S-PC-B138</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2409,7 +2411,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>4001211903</v>
+        <v>4001211902</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2418,24 +2420,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>OR004001211903</t>
+          <t>OR004001211902</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-PRV7700</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-PRV7012</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>DETENDEUR GAZ DE LA BOUTEILLE PROPANNE</t>
+          <t>REGULATEUR PRESSION FUEL ENTRÈE BRULEUR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>S-PC-PRV7700</t>
+          <t>S-PC-PRV7012</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2496,33 +2498,33 @@
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>4001211911</v>
+        <v>4001211903</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>REVISION DETECTEUR DE FLAMME</t>
+          <t>REVISION DETENDEUR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>OR004001211911</t>
+          <t>OR004001211903</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-XY7705</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-PRV7700</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
+          <t>DETENDEUR GAZ DE LA BOUTEILLE PROPANNE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>S-PC-XY7705</t>
+          <t>S-PC-PRV7700</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2583,33 +2585,33 @@
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>4001211913</v>
+        <v>4001211911</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>REVISION FIN DE COURSE</t>
+          <t>REVISION DETECTEUR DE FLAMME</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>OR004001211913</t>
+          <t>OR004001211911</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-ZS7706</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-XY7705</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>FIN DE COURSE DE FERMETURE BRULEUR</t>
+          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>S-PC-ZS7706</t>
+          <t>S-PC-XY7705</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2668,37 +2670,35 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
-        <v>12873778</v>
-      </c>
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>4002021014</v>
+        <v>4001211913</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PREVENTIF SYSTEMATIQUE</t>
+          <t>REVISION FIN DE COURSE</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>OR004002021014</t>
+          <t>OR004001211913</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-REACTI-0CA208-SURV-TI105</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-ZS7706</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SONDE TEMPERATURE PT100 BOUILLET DU CA</t>
+          <t>FIN DE COURSE DE FERMETURE BRULEUR</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>S-PC-TI105</t>
+          <t>S-PC-ZS7706</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2728,21 +2728,21 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>IP1020260601</t>
+          <t>IP1020260209</t>
         </is>
       </c>
       <c r="P26" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>46174</v>
+        <v>46062</v>
       </c>
       <c r="R26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois | Performance Systématiques</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -2752,42 +2752,42 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Respecter l'échéancier des interventions systématiques préventives.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>12873810</v>
+        <v>12073842</v>
       </c>
       <c r="B27" t="n">
-        <v>4002021016</v>
+        <v>4001211955</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PREVENTIF SYSTEMATIQUE</t>
+          <t>Préventif régulation TSP</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>OR004002021016</t>
+          <t>OR004001211955</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-SECHAG-0HB140-SURV-TI140</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-TIC7104</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SONDE TEMP PT100,SORTIE SECHEUR</t>
+          <t>SONDE TEMP K SORTIE  CHAMBRE COMBUS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>S-PC-TI140</t>
+          <t>S-PC-TIC7104</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>LANC ARCO CCRP ERCT RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2817,21 +2817,21 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>IP1020260601</t>
+          <t>IP1020260209</t>
         </is>
       </c>
       <c r="P27" s="2" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>46174</v>
+        <v>46062</v>
       </c>
       <c r="R27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois | Performance Systématiques</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -2841,42 +2841,42 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Respecter l'échéancier des interventions systématiques préventives.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>12873854</v>
+        <v>12873778</v>
       </c>
       <c r="B28" t="n">
-        <v>4002021070</v>
+        <v>4002021014</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Contrôle volet air primaire</t>
+          <t>PREVENTIF SYSTEMATIQUE</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>OR004002021070</t>
+          <t>OR004002021014</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-ZT7403</t>
+          <t>SF01-PE-00LS-REACTI-0CA208-SURV-TI105</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>SERVO ELEC VAN REG DEBIT AIR PRIMAIRE</t>
+          <t>SONDE TEMPERATURE PT100 BOUILLET DU CA</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>S-PC-ZT7403</t>
+          <t>S-PC-TI105</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2910,17 +2910,17 @@
         </is>
       </c>
       <c r="P28" s="2" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="Q28" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="R28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois</t>
+          <t>OT exécution &lt;1 mois | Performance Systématiques</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -2930,16 +2930,16 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Respecter l'échéancier des interventions systématiques préventives.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>12873907</v>
+        <v>12873810</v>
       </c>
       <c r="B29" t="n">
-        <v>4002021143</v>
+        <v>4002021016</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2948,24 +2948,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>OR004002021143</t>
+          <t>OR004002021016</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-REACTI-0CA208-SURV-PT101</t>
+          <t>SF01-PE-00LS-SECHAG-0HB140-SURV-TI140</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TRANSMETTEUR DE PRESSION  VAPEUR ECA</t>
+          <t>SONDE TEMP PT100,SORTIE SECHEUR</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>S-PC-PT101</t>
+          <t>S-PC-TI140</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>LANC CCRP PART RIMP</t>
+          <t>LANC ARCO CCRP ERCT RIMP</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2999,17 +2999,17 @@
         </is>
       </c>
       <c r="P29" s="2" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="Q29" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="R29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois</t>
+          <t>OT exécution &lt;1 mois | Performance Systématiques</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -3019,42 +3019,42 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Respecter l'échéancier des interventions systématiques préventives.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>12873970</v>
+        <v>12873854</v>
       </c>
       <c r="B30" t="n">
-        <v>4002021210</v>
+        <v>4002021070</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Contrôle volet air combustion</t>
+          <t>Contrôle volet air primaire</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>OR004002021210</t>
+          <t>OR004002021070</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-ZT7404</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-ZT7403</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>SERVOM ELEC VOLET AIR DE COMBUSTION</t>
+          <t>SERVO ELEC VAN REG DEBIT AIR PRIMAIRE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>S-PC-ZT7404</t>
+          <t>S-PC-ZT7403</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3088,17 +3088,17 @@
         </is>
       </c>
       <c r="P30" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="Q30" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="R30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois | Performance Systématiques</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -3108,16 +3108,16 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Respecter l'échéancier des interventions systématiques préventives.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>12890928</v>
+        <v>12873907</v>
       </c>
       <c r="B31" t="n">
-        <v>4002037489</v>
+        <v>4002021143</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3126,24 +3126,24 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>OR004002037489</t>
+          <t>OR004002021143</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SF01-PE-FUEL-00SURV-PG7002</t>
+          <t>SF01-PE-00LS-REACTI-0CA208-SURV-PT101</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>MANOMETRE FUEL SORTIE BAC FUEL</t>
+          <t>TRANSMETTEUR DE PRESSION  VAPEUR ECA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>S-PC-PG7002</t>
+          <t>S-PC-PT101</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3173,14 +3173,14 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>IP1020260604</t>
+          <t>IP1020260601</t>
         </is>
       </c>
       <c r="P31" s="2" t="n">
         <v>46291</v>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>46177</v>
+        <v>46174</v>
       </c>
       <c r="R31" t="n">
         <v>1</v>
@@ -3203,36 +3203,36 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>12890982</v>
+        <v>12873970</v>
       </c>
       <c r="B32" t="n">
-        <v>4002037543</v>
+        <v>4002021210</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PREVENTIF SYSTEMATIQUE</t>
+          <t>Contrôle volet air combustion</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>OR004002037543</t>
+          <t>OR004002021210</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SF01-PE-00LN-REACTI-0CA207-SURV-FV209</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-ZT7404</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>VANNE REGULATION DEBIT VAPEUR ENTRÉE CA</t>
+          <t>SERVOM ELEC VOLET AIR DE COMBUSTION</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>S-PC-FV209</t>
+          <t>S-PC-ZT7404</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3262,21 +3262,21 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>IP1020260604</t>
+          <t>IP1020260601</t>
         </is>
       </c>
       <c r="P32" s="2" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>46177</v>
+        <v>46174</v>
       </c>
       <c r="R32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>OT exécution &lt;1 mois</t>
+          <t>OT exécution &lt;1 mois | Performance Systématiques</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -3286,42 +3286,42 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé. | Respecter l'échéancier des interventions systématiques préventives.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>13182917</v>
+        <v>12890928</v>
       </c>
       <c r="B33" t="n">
-        <v>4002310284</v>
+        <v>4002037489</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Contrôle pressostat</t>
+          <t>PREVENTIF SYSTEMATIQUE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>OR004002310284</t>
+          <t>OR004002037489</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SF01-PE-FUEL-00SURV-PH7026</t>
+          <t>SF01-PE-FUEL-00SURV-PG7002</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PRESSOSTAT REFOULEMENT POMPE FUEL HD335B</t>
+          <t>MANOMETRE FUEL SORTIE BAC FUEL</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>S-PC-PSH7026</t>
+          <t>S-PC-PG7002</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3351,14 +3351,14 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>IP1020260714</t>
+          <t>IP1020260604</t>
         </is>
       </c>
       <c r="P33" s="2" t="n">
         <v>46291</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>46217</v>
+        <v>46177</v>
       </c>
       <c r="R33" t="n">
         <v>1</v>
@@ -3381,36 +3381,36 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>10080825</v>
+        <v>12890982</v>
       </c>
       <c r="B34" t="n">
-        <v>4123683</v>
+        <v>4002037543</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>INSTALLATION DEBITMETRE SUR CIRCUIT SOUF</t>
+          <t>PREVENTIF SYSTEMATIQUE</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>OR000004123683</t>
+          <t>OR004002037543</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SF01-PE-00LN-REACTI-0CA207-SURV</t>
+          <t>SF01-PE-00LN-REACTI-0CA207-SURV-FV209</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CONTRÔLE ET SURVIELLANCE</t>
+          <t>VANNE REGULATION DEBIT VAPEUR ENTRÉE CA</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>NOUVEAU PT_SAP</t>
+          <t>S-PC-FV209</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>TCLO CONF IMPR ARCO CCRP ERCT JBFI MMEf*</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -3440,66 +3440,66 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260604</t>
         </is>
       </c>
       <c r="P34" s="2" t="n">
-        <v>45679</v>
+        <v>46291</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>45679</v>
+        <v>46177</v>
       </c>
       <c r="R34" t="n">
         <v>1</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>10082114</v>
+        <v>13182917</v>
       </c>
       <c r="B35" t="n">
-        <v>4124353</v>
+        <v>4002310284</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>installation servomoteur sur circuit con</t>
+          <t>Contrôle pressostat</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>OR000004124353</t>
+          <t>OR004002310284</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SF01-PE-00LN-REACTI-0CA207-SURV</t>
+          <t>SF01-PE-FUEL-00SURV-PH7026</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>CONTRÔLE ET SURVIELLANCE</t>
+          <t>PRESSOSTAT REFOULEMENT POMPE FUEL HD335B</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>NOUVEAU PT_SAP</t>
+          <t>S-PC-PSH7026</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>TCLO CONF IMPR ARCO CCRP ERCT JBFI MMEf*</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3529,66 +3529,66 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260714</t>
         </is>
       </c>
       <c r="P35" s="2" t="n">
-        <v>45681</v>
+        <v>46291</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>45681</v>
+        <v>46217</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>10117792</v>
+        <v>13491439</v>
       </c>
       <c r="B36" t="n">
-        <v>4158428</v>
+        <v>4002585436</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CANGEMENT DET FLAMME LS</t>
+          <t>Inspection 7j de analyseur gaz</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>OR000004158428</t>
+          <t>OR004002585436</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-XY7705</t>
+          <t>SF01-PE-BATI-SLAGHF</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
+          <t>SALLE ANALYSEURS GAZ HF</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>S-PC-XY7705</t>
+          <t>NOUVEAU PT_SAP</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3618,66 +3618,66 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260828</t>
         </is>
       </c>
       <c r="P36" s="2" t="n">
-        <v>45699</v>
+        <v>46292</v>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>45699</v>
+        <v>46262</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>10385897</v>
+        <v>13491406</v>
       </c>
       <c r="B37" t="n">
-        <v>4433877</v>
+        <v>4002585495</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CHANGEMENT TRANSMETTEUR UNIVERSEL LS</t>
+          <t>CONTROLE SYSTEMATIQUE API CAC LN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>OR000004433877</t>
+          <t>OR004002585495</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-ARLC-CONVCORA</t>
+          <t>SF01-PE-00LN-COMBUS-0HD301-ARAU</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CONVERTISSEUR DE COURANT</t>
+          <t>ARMOIRE AUTOMATE CHAMBRE LN</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>NOUVEAU PT_SAP</t>
+          <t>S-PC-API-C-LN</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3707,66 +3707,66 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260828</t>
         </is>
       </c>
       <c r="P37" s="2" t="n">
-        <v>45768</v>
+        <v>46292</v>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>45768</v>
+        <v>46262</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>10384457</v>
+        <v>13491443</v>
       </c>
       <c r="B38" t="n">
-        <v>4433930</v>
+        <v>4002585500</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CHANGEMENT TRANSMETTEUR UNIVERSEL</t>
+          <t>Contrôle détecteur flamme XY7705</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>OR000004433930</t>
+          <t>OR004002585500</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SF01-PE-00LN-COMBUS-0HD301-SURV</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-XY7705</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CONTRÔLE ET SURVEILLANCE</t>
+          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>NOUVEAU PT_SAP</t>
+          <t>S-PC-XY7705</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3796,66 +3796,66 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260828</t>
         </is>
       </c>
       <c r="P38" s="2" t="n">
-        <v>45768</v>
+        <v>46292</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>45768</v>
+        <v>46262</v>
       </c>
       <c r="R38" t="n">
         <v>1</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>10485278</v>
+        <v>13491479</v>
       </c>
       <c r="B39" t="n">
-        <v>4544446</v>
+        <v>4002585516</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CHANGEMENT SONDE TEMPERATEUR</t>
+          <t>Contrôle détecteur flamme XY LN</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>OR000004544446</t>
+          <t>OR004002585516</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SF01-PE-00LN-COMBUS-0HD301-SURV-TIC3017</t>
+          <t>SF01-PE-00LN-COMBUS-0HD301-SURV-XY3705</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>SONDE TEMP PT100 FUEL SORTIE RECHAUF</t>
+          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>S-PC-TIC3017</t>
+          <t>S-PC-XY3705</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3885,66 +3885,66 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260828</t>
         </is>
       </c>
       <c r="P39" s="2" t="n">
-        <v>45791</v>
+        <v>46292</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>45791</v>
+        <v>46262</v>
       </c>
       <c r="R39" t="n">
         <v>1</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>10601031</v>
+        <v>13491451</v>
       </c>
       <c r="B40" t="n">
-        <v>4673659</v>
+        <v>4002585520</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CHANGEMENT VANNE FUEL LS</t>
+          <t>CONTROLE SYSTEMATIQUE API CAC LS</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>OR000004673659</t>
+          <t>OR004002585520</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-TV7613</t>
+          <t>SF01-PE-00LS-COMBUS-0HD302-ARAU</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>VAN VAP REG TEMP DU RECHAUFFEUR FUEL</t>
+          <t>ARMOIRE AUTOMATE CHAMBRE LS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>S-PC-TV7613</t>
+          <t>S-PC-API-C-LS</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>TCLO CONF ARCO CCRP JBFI MMEf RIMP</t>
+          <t>LANC CCRP PART RIMP</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3974,29 +3974,1364 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>DOUIOUI</t>
+          <t>IP1020260828</t>
         </is>
       </c>
       <c r="P40" s="2" t="n">
-        <v>45810</v>
+        <v>46292</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>45810</v>
+        <v>46262</v>
       </c>
       <c r="R40" t="n">
         <v>1</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>13491454</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4002585523</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CONTROLE SYSTEMATIQUE DOSO LS TSP</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>OR004002585523</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-REACTI-0HA042-SURV</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVEILLANCE</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R41" t="n">
+        <v>1</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>13491459</v>
+      </c>
+      <c r="B42" t="n">
+        <v>4002585528</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>RONDE INSPECTION DOSO LS</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>OR004002585528</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-REACTI-0HA042-SURV</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVEILLANCE</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>13491502</v>
+      </c>
+      <c r="B43" t="n">
+        <v>4002585531</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>RONDE INSPECTION DOSO LN</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>OR004002585531</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-REACTI-0HA041-SURV</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVIELLANCE</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>CRPR ATPL SOPL</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R43" t="n">
+        <v>1</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>13491429</v>
+      </c>
+      <c r="B44" t="n">
+        <v>4002585540</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PREVENTIF SYSTEMATIQUE BAS PF LS</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>OR004002585540</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-TRANPF-0IA067-W107</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>BASCULE INTEGRATRICE DU PRODUIT FINI LS</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>S-PC-WIQ107</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R44" t="n">
+        <v>1</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>13491480</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4002585551</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PREVENTIF SYSTEMATIQUE BAS RECY LN</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>OR004002585551</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-TRRECY-0HA033-BASC</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>BASCULE</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>13491486</v>
+      </c>
+      <c r="B46" t="n">
+        <v>4002585557</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PREVENTIF SYSTEMATIQUE BAS PF LN</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>OR004002585557</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-TRANPF-0IA029-W207</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>BASCULE INTEGRATRICE DU PRODUIT FINI LN</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>S-PC-WIQ207</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>13491489</v>
+      </c>
+      <c r="B47" t="n">
+        <v>4002585560</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PEVENTIF 7J INSTRUM CAC LN</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>OR004002585560</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-COMBUS-0HD301</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>CHAMBRE A COMBUSTION HD301 LIGNE NORD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>S-PC-HD301</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R47" t="n">
+        <v>1</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>13491512</v>
+      </c>
+      <c r="B48" t="n">
+        <v>4002585563</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CONTROLE SYSTEMATIQUE INSTRUM CAC LS</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>OR004002585563</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-COMBUS-0HD302</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>CHAMBRE A COMBUSTION HD302 LIGNE SUD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>S-PC-HD302</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>IP1020260828</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="R48" t="n">
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>10080825</v>
+      </c>
+      <c r="B49" t="n">
+        <v>4123683</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>INSTALLATION DEBITMETRE SUR CIRCUIT SOUF</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>OR000004123683</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-REACTI-0CA207-SURV</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVIELLANCE</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>TCLO CONF IMPR ARCO CCRP ERCT JBFI MMEf*</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>45679</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>45679</v>
+      </c>
+      <c r="R49" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
           <t>OT_COR_EGAL</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr">
+      <c r="T49" t="inlineStr">
         <is>
           <t>Agent de Saisie</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>10082114</v>
+      </c>
+      <c r="B50" t="n">
+        <v>4124353</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>installation servomoteur sur circuit con</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>OR000004124353</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-REACTI-0CA207-SURV</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVIELLANCE</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>TCLO CONF IMPR ARCO CCRP ERCT JBFI MMEf*</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>45681</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>45681</v>
+      </c>
+      <c r="R50" t="n">
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>10117792</v>
+      </c>
+      <c r="B51" t="n">
+        <v>4158428</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CANGEMENT DET FLAMME LS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>OR000004158428</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-XY7705</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>S-PC-XY7705</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>45699</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>45699</v>
+      </c>
+      <c r="R51" t="n">
+        <v>1</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>10385897</v>
+      </c>
+      <c r="B52" t="n">
+        <v>4433877</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CHANGEMENT TRANSMETTEUR UNIVERSEL LS</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>OR000004433877</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-COMBUS-0HD302-ARLC-CONVCORA</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>CONVERTISSEUR DE COURANT</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>45768</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>45768</v>
+      </c>
+      <c r="R52" t="n">
+        <v>1</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>10384457</v>
+      </c>
+      <c r="B53" t="n">
+        <v>4433930</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CHANGEMENT TRANSMETTEUR UNIVERSEL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>OR000004433930</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-COMBUS-0HD301-SURV</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVEILLANCE</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="n">
+        <v>45768</v>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>45768</v>
+      </c>
+      <c r="R53" t="n">
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>10485278</v>
+      </c>
+      <c r="B54" t="n">
+        <v>4544446</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CHANGEMENT SONDE TEMPERATEUR</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>OR000004544446</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LN-COMBUS-0HD301-SURV-TIC3017</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SONDE TEMP PT100 FUEL SORTIE RECHAUF</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>S-PC-TIC3017</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>TCLO CONF ARCO CCRP ERCT JBFI MMEf RIMP</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>45791</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>45791</v>
+      </c>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>10601031</v>
+      </c>
+      <c r="B55" t="n">
+        <v>4673659</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CHANGEMENT VANNE FUEL LS</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>OR000004673659</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SF01-PE-00LS-COMBUS-0HD302-SURV-TV7613</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>VAN VAP REG TEMP DU RECHAUFFEUR FUEL</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>S-PC-TV7613</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>SF1-RTSP</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>TCLO CONF ARCO CCRP JBFI MMEf RIMP</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>DOUIOUI</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>45810</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>45810</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
         <is>
           <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
         </is>

</xml_diff>